<commit_message>
feat(gui): add custom multimeter application icon
Add application icon with multiple resolutions (16x16 to 256x256) and integrate it into the build process. The icon now appears in the window title bar and taskbar, improving application visibility and user experience.

Changes include:
- Added app_icon.ico and PNG source files at various resolutions
- Updated PyInstaller spec to embed icon in executable
- Modified build script to verify icon existence before build
- Enhanced icon setting in main.py and gui/window.py with debug logging
- Bumped version to 1.7.1
</commit_message>
<xml_diff>
--- a/Boreas_2v1_2026-01-30_3.xlsx
+++ b/Boreas_2v1_2026-01-30_3.xlsx
@@ -1,53 +1,92 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="22026"/>
   <workbookPr/>
-  <workbookProtection/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\NextCloud\pythonProject\SDM4055A_Controller\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3736AADD-AC83-4A87-8836-8C9499F9B727}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView xWindow="30612" yWindow="-108" windowWidth="30936" windowHeight="16896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Report" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Report" sheetId="1" r:id="rId1"/>
   </sheets>
-  <definedNames/>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
+  <si>
+    <t>QR</t>
+  </si>
+  <si>
+    <t>TEST RESULT</t>
+  </si>
+  <si>
+    <t>CH1 (12.0V)</t>
+  </si>
+  <si>
+    <t>CH2 (5.0V)</t>
+  </si>
+  <si>
+    <t>CH3 (3.3V)</t>
+  </si>
+  <si>
+    <t>Date/Time</t>
+  </si>
+  <si>
+    <t>PSN000006047</t>
+  </si>
+  <si>
+    <t>FAILED CH1 (12.0V): -0.0003873 (expected: 11.5 - 12.5); CH2 (5.0V): -0.0003633 (expected: 4.9 - 5.1); CH3 (3.3V): 0.0617449 (expected: 2.95 - 3.05)</t>
+  </si>
+  <si>
+    <t>-0.0003873</t>
+  </si>
+  <si>
+    <t>-0.0003633</t>
+  </si>
+  <si>
+    <t>0.0617449</t>
+  </si>
+  <si>
+    <t>2026-01-30 17:29:57</t>
+  </si>
+</sst>
+</file>
+
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
-  <fonts count="2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
-      <color theme="1"/>
-      <sz val="11"/>
       <scheme val="minor"/>
     </font>
     <font>
+      <b/>
+      <sz val="11"/>
       <name val="Arial"/>
-      <b val="1"/>
-      <sz val="11"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="3">
     <fill>
-      <patternFill/>
+      <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00CCFFCC"/>
-        <bgColor rgb="00CCFFCC"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FFCCCC"/>
-        <bgColor rgb="00FFCCCC"/>
+        <fgColor rgb="FFFFCCCC"/>
+        <bgColor rgb="FFFFCCCC"/>
       </patternFill>
     </fill>
   </fills>
@@ -61,103 +100,44 @@
     </border>
     <border>
       <left style="thin">
-        <color rgb="00000000"/>
+        <color rgb="FF000000"/>
       </left>
       <right style="thin">
-        <color rgb="00000000"/>
+        <color rgb="FF000000"/>
       </right>
       <top style="thin">
-        <color rgb="00000000"/>
+        <color rgb="FF000000"/>
       </top>
       <bottom style="thin">
-        <color rgb="00000000"/>
+        <color rgb="FF000000"/>
       </bottom>
+      <diagonal/>
     </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+  <cellXfs count="4">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+    <cellStyle name="Обычный" xfId="0" builtinId="0"/>
   </cellStyles>
+  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
-  <colors>
-    <indexedColors>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008000"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00808000"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="00C0C0C0"/>
-      <rgbColor rgb="00808080"/>
-      <rgbColor rgb="009999FF"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00FFFFCC"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00660066"/>
-      <rgbColor rgb="00FF8080"/>
-      <rgbColor rgb="000066CC"/>
-      <rgbColor rgb="00CCCCFF"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="0000CCFF"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00CCFFCC"/>
-      <rgbColor rgb="00FFFF99"/>
-      <rgbColor rgb="0099CCFF"/>
-      <rgbColor rgb="00FF99CC"/>
-      <rgbColor rgb="00CC99FF"/>
-      <rgbColor rgb="00FFCC99"/>
-      <rgbColor rgb="003366FF"/>
-      <rgbColor rgb="0033CCCC"/>
-      <rgbColor rgb="0099CC00"/>
-      <rgbColor rgb="00FFCC00"/>
-      <rgbColor rgb="00FF9900"/>
-      <rgbColor rgb="00FF6600"/>
-      <rgbColor rgb="00666699"/>
-      <rgbColor rgb="00969696"/>
-      <rgbColor rgb="00003366"/>
-      <rgbColor rgb="00339966"/>
-      <rgbColor rgb="00003300"/>
-      <rgbColor rgb="00333300"/>
-      <rgbColor rgb="00993300"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00333399"/>
-      <rgbColor rgb="00333333"/>
-    </indexedColors>
-  </colors>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
@@ -445,84 +425,55 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:F2"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="55" customWidth="1" min="2" max="2"/>
-    <col width="13" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
-    <col width="21" customWidth="1" min="6" max="6"/>
+    <col min="1" max="1" width="14" customWidth="1"/>
+    <col min="2" max="2" width="71.88671875" customWidth="1"/>
+    <col min="3" max="3" width="13" customWidth="1"/>
+    <col min="4" max="5" width="12" customWidth="1"/>
+    <col min="6" max="6" width="21" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>QR</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>TEST RESULT</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>CH1 (12.0V)</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>CH2 (5.0V)</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>CH3 (3.3V)</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>Date/Time</t>
-        </is>
+    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>PSN000006047</t>
-        </is>
-      </c>
-      <c r="B2" s="2" t="inlineStr">
-        <is>
-          <t>FAILED CH3 (3.3V): -3.2983124 (expected: 2.95 - 3.05)</t>
-        </is>
-      </c>
-      <c r="C2" s="3" t="inlineStr">
-        <is>
-          <t>12.1252649</t>
-        </is>
-      </c>
-      <c r="D2" s="3" t="inlineStr">
-        <is>
-          <t>5.0433129</t>
-        </is>
-      </c>
-      <c r="E2" s="4" t="inlineStr">
-        <is>
-          <t>-3.2983124</t>
-        </is>
-      </c>
-      <c r="F2" s="2" t="inlineStr">
-        <is>
-          <t>2026-01-30 17:15:29</t>
-        </is>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A2" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="D2" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="E2" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>11</v>
       </c>
     </row>
   </sheetData>

</xml_diff>